<commit_message>
subiendo para arrancar septiembre
</commit_message>
<xml_diff>
--- a/2026/BELTRAN 34/Desglose de deuda local.xlsx
+++ b/2026/BELTRAN 34/Desglose de deuda local.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\2026\BELTRAN 34\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B61807A-371C-4E3D-B7F4-8A3E902C5791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395CC04E-D96F-4350-B3EC-56A51CDEC3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{40F7CB68-AA62-4B90-B02B-2F8168283C84}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$E$4:$K$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$E$4:$K$93</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="9">
   <si>
     <t>DESGLOSE DEUDA - UF 1 - Local 1/ Entrep. - BELTRAN 34</t>
   </si>
@@ -55,27 +55,6 @@
   </si>
   <si>
     <t>TOTAL:</t>
-  </si>
-  <si>
-    <t>PLAN DE PAGO - OPCIONES:</t>
-  </si>
-  <si>
-    <t>OPCION A)</t>
-  </si>
-  <si>
-    <t>1 CUOTA DE $1.759.317,12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPCION B) </t>
-  </si>
-  <si>
-    <t>2 CUOTAS DE $932.438,07 (TOTAL $1.864.876,14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPCION C) </t>
-  </si>
-  <si>
-    <t>3 CUOTAS DE $639.218,51 (TOTAL $1.917.655,55)</t>
   </si>
 </sst>
 </file>
@@ -117,7 +96,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -136,24 +115,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -168,7 +129,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -180,13 +141,7 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -202,6 +157,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -522,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A0868C-F56B-4272-A7E5-AB78808DF362}">
-  <dimension ref="C4:K84"/>
+  <dimension ref="C4:K93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.5546875" customWidth="1"/>
@@ -533,28 +491,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
     </row>
     <row r="6" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I6" s="10"/>
+      <c r="F6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="7"/>
       <c r="K6" t="s">
         <v>4</v>
       </c>
@@ -563,14 +521,14 @@
       <c r="E7" s="1">
         <v>45658</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="8">
         <v>43440</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12">
+      <c r="G7" s="8"/>
+      <c r="H7" s="8">
         <v>23892</v>
       </c>
-      <c r="I7" s="12"/>
+      <c r="I7" s="8"/>
       <c r="K7" s="3">
         <f>(F7+H7)*3%</f>
         <v>2019.96</v>
@@ -580,14 +538,14 @@
       <c r="E10" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I10" s="10"/>
+      <c r="F10" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7"/>
       <c r="K10" t="s">
         <v>4</v>
       </c>
@@ -597,14 +555,14 @@
         <f>E7+31</f>
         <v>45689</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="8">
         <v>54300</v>
       </c>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12">
+      <c r="G11" s="8"/>
+      <c r="H11" s="8">
         <v>23892</v>
       </c>
-      <c r="I11" s="12"/>
+      <c r="I11" s="8"/>
       <c r="K11" s="3">
         <f>(F11+H11)*3%</f>
         <v>2345.7599999999998</v>
@@ -614,14 +572,14 @@
       <c r="E14" t="s">
         <v>1</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I14" s="10"/>
+      <c r="F14" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14" s="7"/>
       <c r="K14" t="s">
         <v>4</v>
       </c>
@@ -631,14 +589,14 @@
         <f>E11+31</f>
         <v>45720</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="8">
         <v>70590</v>
       </c>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12">
+      <c r="G15" s="8"/>
+      <c r="H15" s="8">
         <v>23892</v>
       </c>
-      <c r="I15" s="12"/>
+      <c r="I15" s="8"/>
       <c r="K15" s="3">
         <f>(F15+H15)*3%</f>
         <v>2834.46</v>
@@ -648,14 +606,14 @@
       <c r="E18" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I18" s="10"/>
+      <c r="F18" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I18" s="7"/>
       <c r="K18" t="s">
         <v>4</v>
       </c>
@@ -665,12 +623,12 @@
         <f>E15+31</f>
         <v>45751</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="8">
         <v>86880</v>
       </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
       <c r="K19" s="3">
         <f>(F19+H19)*3%</f>
         <v>2606.4</v>
@@ -680,14 +638,14 @@
       <c r="E22" t="s">
         <v>1</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I22" s="10"/>
+      <c r="F22" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="7"/>
       <c r="K22" t="s">
         <v>4</v>
       </c>
@@ -697,12 +655,12 @@
         <f>E19+31</f>
         <v>45782</v>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="8">
         <v>86880</v>
       </c>
-      <c r="G23" s="12"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
       <c r="K23" s="3">
         <f>(F23+H23)*3%</f>
         <v>2606.4</v>
@@ -712,14 +670,14 @@
       <c r="E26" t="s">
         <v>1</v>
       </c>
-      <c r="F26" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I26" s="11"/>
+      <c r="F26" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="I26" s="13"/>
       <c r="K26" t="s">
         <v>4</v>
       </c>
@@ -729,12 +687,12 @@
         <f>E23+31</f>
         <v>45813</v>
       </c>
-      <c r="F27" s="17">
+      <c r="F27" s="14">
         <v>97740</v>
       </c>
-      <c r="G27" s="17"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
       <c r="K27" s="3">
         <f>(F27+H27)*3%</f>
         <v>2932.2</v>
@@ -744,14 +702,14 @@
       <c r="E30" t="s">
         <v>1</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I30" s="10"/>
+      <c r="F30" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I30" s="7"/>
       <c r="K30" t="s">
         <v>4</v>
       </c>
@@ -761,12 +719,12 @@
         <f>E27+31</f>
         <v>45844</v>
       </c>
-      <c r="F31" s="12">
+      <c r="F31" s="8">
         <v>55903.81</v>
       </c>
-      <c r="G31" s="12"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
       <c r="K31" s="3">
         <f>(F31+H31)*3%</f>
         <v>1677.1143</v>
@@ -782,14 +740,14 @@
       <c r="E34" t="s">
         <v>1</v>
       </c>
-      <c r="F34" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I34" s="11"/>
+      <c r="F34" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="I34" s="13"/>
       <c r="K34" t="s">
         <v>4</v>
       </c>
@@ -799,12 +757,12 @@
         <f>E31+31</f>
         <v>45875</v>
       </c>
-      <c r="F35" s="17">
+      <c r="F35" s="14">
         <v>124890</v>
       </c>
-      <c r="G35" s="17"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
       <c r="K35" s="3">
         <f>(F35+H35)*3%</f>
         <v>3746.7</v>
@@ -814,14 +772,14 @@
       <c r="E38" t="s">
         <v>1</v>
       </c>
-      <c r="F38" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I38" s="11"/>
+      <c r="F38" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="I38" s="13"/>
       <c r="K38" t="s">
         <v>4</v>
       </c>
@@ -831,10 +789,10 @@
         <f>E35+31</f>
         <v>45906</v>
       </c>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
       <c r="K39" s="3">
         <f>(F39+H39)*3%</f>
         <v>0</v>
@@ -844,14 +802,14 @@
       <c r="E42" t="s">
         <v>1</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I42" s="10"/>
+      <c r="F42" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I42" s="7"/>
       <c r="K42" t="s">
         <v>4</v>
       </c>
@@ -861,12 +819,12 @@
         <f>E39+31</f>
         <v>45937</v>
       </c>
-      <c r="F43" s="12">
+      <c r="F43" s="8">
         <v>106428</v>
       </c>
-      <c r="G43" s="12"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="10"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
       <c r="K43" s="3">
         <f>(F43+H43)*3%</f>
         <v>3192.8399999999997</v>
@@ -876,14 +834,14 @@
       <c r="E46" t="s">
         <v>1</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I46" s="10"/>
+      <c r="F46" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I46" s="7"/>
       <c r="K46" t="s">
         <v>4</v>
       </c>
@@ -893,12 +851,12 @@
         <f>E43+31</f>
         <v>45968</v>
       </c>
-      <c r="F47" s="12">
+      <c r="F47" s="8">
         <v>157470</v>
       </c>
-      <c r="G47" s="12"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
       <c r="K47" s="3">
         <f>(F47+H47)*3%</f>
         <v>4724.0999999999995</v>
@@ -908,14 +866,14 @@
       <c r="E50" t="s">
         <v>1</v>
       </c>
-      <c r="F50" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I50" s="10"/>
+      <c r="F50" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I50" s="7"/>
       <c r="K50" t="s">
         <v>4</v>
       </c>
@@ -925,12 +883,12 @@
         <f>E47+31</f>
         <v>45999</v>
       </c>
-      <c r="F51" s="12">
+      <c r="F51" s="8">
         <v>195480</v>
       </c>
-      <c r="G51" s="12"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
       <c r="K51" s="3">
         <f>(F51+H51)*3%</f>
         <v>5864.4</v>
@@ -940,14 +898,14 @@
       <c r="E54" t="s">
         <v>1</v>
       </c>
-      <c r="F54" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I54" s="10"/>
+      <c r="F54" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I54" s="7"/>
       <c r="K54" t="s">
         <v>4</v>
       </c>
@@ -957,14 +915,14 @@
         <f>E51+31</f>
         <v>46030</v>
       </c>
-      <c r="F55" s="12">
+      <c r="F55" s="8">
         <v>152730.859986</v>
       </c>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12">
+      <c r="G55" s="8"/>
+      <c r="H55" s="8">
         <v>1194.5999999999999</v>
       </c>
-      <c r="I55" s="12"/>
+      <c r="I55" s="8"/>
       <c r="K55" s="3">
         <f>(F55+H55)*3%</f>
         <v>4617.7637995799996</v>
@@ -990,14 +948,14 @@
       <c r="E58" t="s">
         <v>1</v>
       </c>
-      <c r="F58" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I58" s="10"/>
+      <c r="F58" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I58" s="7"/>
       <c r="K58" t="s">
         <v>4</v>
       </c>
@@ -1007,14 +965,14 @@
         <f>E55+31</f>
         <v>46061</v>
       </c>
-      <c r="F59" s="12">
+      <c r="F59" s="8">
         <v>184619.99999999997</v>
       </c>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12">
+      <c r="G59" s="8"/>
+      <c r="H59" s="8">
         <v>2280.6</v>
       </c>
-      <c r="I59" s="12"/>
+      <c r="I59" s="8"/>
       <c r="K59" s="3">
         <f>(F59+H59)*3%</f>
         <v>5607.0179999999991</v>
@@ -1040,14 +998,14 @@
       <c r="E62" t="s">
         <v>1</v>
       </c>
-      <c r="F62" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I62" s="10"/>
+      <c r="F62" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I62" s="7"/>
       <c r="K62" t="s">
         <v>4</v>
       </c>
@@ -1057,14 +1015,14 @@
         <f>E59+31</f>
         <v>46092</v>
       </c>
-      <c r="F63" s="12">
+      <c r="F63" s="8">
         <v>212312.99999999997</v>
       </c>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12">
+      <c r="G63" s="8"/>
+      <c r="H63" s="8">
         <v>3257.9999999999995</v>
       </c>
-      <c r="I63" s="12"/>
+      <c r="I63" s="8"/>
       <c r="K63" s="3">
         <f>(F63+H63)*3%</f>
         <v>6467.1299999999992</v>
@@ -1090,14 +1048,14 @@
       <c r="E66" t="s">
         <v>1</v>
       </c>
-      <c r="F66" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G66" s="10"/>
-      <c r="H66" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I66" s="10"/>
+      <c r="F66" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I66" s="7"/>
       <c r="K66" t="s">
         <v>4</v>
       </c>
@@ -1107,14 +1065,14 @@
         <f>E63+31</f>
         <v>46123</v>
       </c>
-      <c r="F67" s="12">
+      <c r="F67" s="8">
         <v>212313</v>
       </c>
-      <c r="G67" s="12"/>
-      <c r="H67" s="12">
+      <c r="G67" s="8"/>
+      <c r="H67" s="8">
         <v>0</v>
       </c>
-      <c r="I67" s="12"/>
+      <c r="I67" s="8"/>
       <c r="K67" s="3">
         <f>(F67+H67)*3%</f>
         <v>6369.3899999999994</v>
@@ -1140,14 +1098,14 @@
       <c r="E70" t="s">
         <v>1</v>
       </c>
-      <c r="F70" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I70" s="10"/>
+      <c r="F70" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G70" s="7"/>
+      <c r="H70" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I70" s="7"/>
       <c r="K70" t="s">
         <v>4</v>
       </c>
@@ -1157,15 +1115,15 @@
         <f>E67+31</f>
         <v>46154</v>
       </c>
-      <c r="F71" s="12">
+      <c r="F71" s="8">
         <f>F67</f>
         <v>212313</v>
       </c>
-      <c r="G71" s="12"/>
-      <c r="H71" s="12">
+      <c r="G71" s="8"/>
+      <c r="H71" s="8">
         <v>61359</v>
       </c>
-      <c r="I71" s="12"/>
+      <c r="I71" s="8"/>
       <c r="K71" s="3">
         <f>(F71+H71)*3%</f>
         <v>8210.16</v>
@@ -1187,136 +1145,245 @@
       <c r="I73" s="6"/>
       <c r="K73" s="3"/>
     </row>
-    <row r="74" spans="5:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E74" t="s">
+        <v>1</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G74" s="7"/>
+      <c r="H74" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I74" s="7"/>
+      <c r="K74" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E75" s="1">
+        <f>E71+31</f>
+        <v>46185</v>
+      </c>
+      <c r="F75" s="8">
+        <v>178848</v>
+      </c>
+      <c r="G75" s="8"/>
+      <c r="H75" s="8">
+        <v>148000</v>
+      </c>
+      <c r="I75" s="8"/>
+      <c r="K75" s="3">
+        <f>(F75+H75)*3%</f>
+        <v>9805.44</v>
+      </c>
+    </row>
+    <row r="76" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E76" s="1"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6"/>
+      <c r="H76" s="6"/>
+      <c r="I76" s="6"/>
+      <c r="K76" s="3"/>
+    </row>
+    <row r="77" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E77" s="1"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="6"/>
+      <c r="H77" s="6"/>
+      <c r="I77" s="6"/>
+      <c r="K77" s="3"/>
+    </row>
+    <row r="78" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E78" t="s">
+        <v>1</v>
+      </c>
+      <c r="F78" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G78" s="7"/>
+      <c r="H78" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I78" s="7"/>
+      <c r="K78" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E79" s="1">
+        <f>E75+31</f>
+        <v>46216</v>
+      </c>
+      <c r="F79" s="8">
+        <v>178848</v>
+      </c>
+      <c r="G79" s="8"/>
+      <c r="H79" s="8">
+        <v>75000</v>
+      </c>
+      <c r="I79" s="8"/>
+      <c r="K79" s="3">
+        <f>(F79+H79)*3%</f>
+        <v>7615.44</v>
+      </c>
+    </row>
+    <row r="80" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E80" s="1"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="6"/>
+      <c r="H80" s="6"/>
+      <c r="I80" s="6"/>
+      <c r="K80" s="3"/>
+    </row>
+    <row r="81" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E81" s="1"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6"/>
+      <c r="K81" s="3"/>
+    </row>
+    <row r="82" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E82" t="s">
+        <v>1</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G82" s="7"/>
+      <c r="H82" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I82" s="7"/>
+      <c r="K82" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E83" s="1">
+        <f>E79+31</f>
+        <v>46247</v>
+      </c>
+      <c r="F83" s="8">
+        <v>163831.62075599999</v>
+      </c>
+      <c r="G83" s="8"/>
+      <c r="H83" s="8">
+        <v>75000</v>
+      </c>
+      <c r="I83" s="8"/>
+      <c r="K83" s="3">
+        <f>(F83+H83)*3%</f>
+        <v>7164.9486226799991</v>
+      </c>
+    </row>
+    <row r="84" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E84" s="1"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
+      <c r="H84" s="6"/>
+      <c r="I84" s="6"/>
+      <c r="K84" s="3"/>
+    </row>
+    <row r="85" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E85" s="1"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="6"/>
+      <c r="H85" s="6"/>
+      <c r="I85" s="6"/>
+      <c r="K85" s="3"/>
+    </row>
+    <row r="86" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E86" s="1"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6"/>
+      <c r="H86" s="6"/>
+      <c r="I86" s="6"/>
+      <c r="K86" s="3"/>
+    </row>
+    <row r="87" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E87" s="1"/>
+      <c r="F87" s="6"/>
+      <c r="G87" s="6"/>
+      <c r="H87" s="6"/>
+      <c r="I87" s="6"/>
+      <c r="K87" s="3"/>
+    </row>
+    <row r="88" spans="5:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E88" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E75" t="s">
+    <row r="89" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E89" t="s">
         <v>6</v>
       </c>
-      <c r="H75" s="10" t="s">
+      <c r="H89" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I75" s="10"/>
-      <c r="J75" s="10"/>
-      <c r="K75" s="10"/>
-    </row>
-    <row r="76" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E76" s="13">
-        <f>F7+H7+H11+F11+F15+H15+H19+F19+F23+H23+H27+F27+F31+H35+F35+H32+H31+H39+F39+F43+H43+H47+F47+F51+H51+F55+H55+F59+H59+F63+H63+F67+H67+F71+H71</f>
-        <v>2194059.8699860005</v>
-      </c>
-      <c r="F76" s="13"/>
-      <c r="G76" s="13"/>
-      <c r="H76" s="13">
-        <f>SUM(K7:K72)</f>
-        <v>65821.796099579995</v>
-      </c>
-      <c r="I76" s="14"/>
-      <c r="J76" s="14"/>
-    </row>
-    <row r="78" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="G78" s="4" t="s">
+      <c r="I89" s="7"/>
+      <c r="J89" s="7"/>
+      <c r="K89" s="7"/>
+    </row>
+    <row r="90" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="E90" s="9">
+        <f>F7+H7+H11+F11+F15+H15+H19+F19+F23+H23+H27+F27+F31+H35+F35+H32+H31+H39+F39+F43+H43+H47+F47+F51+H51+F55+H55+F59+H59+F63+H63+F67+H67+F71+H71+F75+F79+H79+H75+F83+H83</f>
+        <v>3013587.4907420003</v>
+      </c>
+      <c r="F90" s="9"/>
+      <c r="G90" s="9"/>
+      <c r="H90" s="9">
+        <f>SUM(K7:K86)</f>
+        <v>90407.624722259992</v>
+      </c>
+      <c r="I90" s="10"/>
+      <c r="J90" s="10"/>
+    </row>
+    <row r="92" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="G92" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="G79" s="15">
-        <f>E76+H76</f>
-        <v>2259881.6660855804</v>
-      </c>
-      <c r="H79" s="15"/>
-      <c r="I79" s="15"/>
-    </row>
-    <row r="81" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E81" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="82" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E82" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F82" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G82" s="7"/>
-      <c r="H82" s="7"/>
-      <c r="I82" s="7"/>
-      <c r="J82" s="7"/>
-      <c r="K82" s="7"/>
-    </row>
-    <row r="83" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E83" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F83" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G83" s="8"/>
-      <c r="H83" s="8"/>
-      <c r="I83" s="8"/>
-      <c r="J83" s="8"/>
-      <c r="K83" s="8"/>
-    </row>
-    <row r="84" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E84" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F84" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G84" s="9"/>
-      <c r="H84" s="9"/>
-      <c r="I84" s="9"/>
-      <c r="J84" s="9"/>
-      <c r="K84" s="9"/>
+    <row r="93" spans="5:11" x14ac:dyDescent="0.3">
+      <c r="G93" s="11">
+        <f>E90+H90</f>
+        <v>3103995.1154642603</v>
+      </c>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="73">
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="H66:I66"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="H67:I67"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="H62:I62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:I63"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="H55:I55"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="H75:K75"/>
-    <mergeCell ref="H76:J76"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="E4:K4"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F43:G43"/>
+  <mergeCells count="85">
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="H83:I83"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="H79:I79"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="H82:I82"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="H74:I74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="H78:I78"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H27:I27"/>
     <mergeCell ref="F47:G47"/>
     <mergeCell ref="F51:G51"/>
     <mergeCell ref="H6:I6"/>
@@ -1333,22 +1400,47 @@
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="H42:I42"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="E90:G90"/>
+    <mergeCell ref="H89:K89"/>
+    <mergeCell ref="H90:J90"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="H55:I55"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:I63"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="H70:I70"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="H67:I67"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>